<commit_message>
design: diseño de los campos de las imagenes
</commit_message>
<xml_diff>
--- a/EJEMPLO/Datos CSV.xlsx
+++ b/EJEMPLO/Datos CSV.xlsx
@@ -3,11 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Excell" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="Excel" sheetId="1" r:id="rId4"/>
     <sheet state="visible" name="CSV" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Excell!$A$1:$Q$31</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Excel!$A$1:$Q$31</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
@@ -96,7 +96,7 @@
     <t>Malbec / Cabernet Sauvignon</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Achaval%20Ferrer%20Quimera.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Achaval_Ferrer_Quimera-removebg-preview.avif</t>
   </si>
   <si>
     <t>activo</t>
@@ -114,7 +114,7 @@
     <t>Malbec</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Catena%20Zapata%20Adrianna%20Vineyard%20Malbec.png</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Catena_Zapata_Adrianna_Vineyard_Malbec-removebg-preview.avif</t>
   </si>
   <si>
     <t>Catena Zapata White Bones Chardonnay</t>
@@ -129,7 +129,7 @@
     <t>Chardonnay</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Catena%20Zapata%20White%20Bones%20Chardonnay.png</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Catena_Zapata_White_Bones_Chardonnay-removebg-preview.avif</t>
   </si>
   <si>
     <t>Chateau Mouton Rothschild</t>
@@ -168,7 +168,7 @@
     <t>Sauvignon Blanc</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Cloudy%20Bay%20Sauvignon%20Blanc.jpeg</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Cloudy_Bay_Sauvignon_Blanc-removebg-preview.avif</t>
   </si>
   <si>
     <t>Concha y Toro Amelia Chardonnay</t>
@@ -186,7 +186,7 @@
     <t>Valle de Casablanca</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Concha%20y%20Toro%20Amelia%20Chardonnay.jpeg</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Concha_y_Toro_Amelia_Chardonnay-removebg-preview.avif</t>
   </si>
   <si>
     <t>Concha y Toro Don Melchor Cabernet Sauvignon</t>
@@ -201,7 +201,7 @@
     <t>Cabernet Sauvignon</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Concha%20y%20Toro%20Don%20Melchor%20Cabernet%20Sauvignon.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Concha_y_Toro_Don_Melchor_Cabernet_Sauvignon-removebg-preview.avif</t>
   </si>
   <si>
     <t>Don Julio Blanco Tequila</t>
@@ -228,7 +228,7 @@
     <t>Agave Azul</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Don%20Julio%20Blanco%20Tequila.jpg</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Don_Julio_Blanco_Tequila-removebg-preview.avif</t>
   </si>
   <si>
     <t>Familia Zuccardi Blanc de Blancs</t>
@@ -246,7 +246,7 @@
     <t>Torrontes / Chardonnay</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Familia%20Zuccardi%20Blanc%20de%20Blancs.jpeg</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Familia_Zuccardi_Blanc_de_Blancs-removebg-preview.avif</t>
   </si>
   <si>
     <t>Flor de Cana 12 anos</t>
@@ -270,7 +270,7 @@
     <t>Ron anejo</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Flor%20de%20Cana%2012%20anos.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Flor_de_Cana_12_anos-removebg-preview.avif</t>
   </si>
   <si>
     <t>Freixenet Cordon Negro Brut</t>
@@ -294,7 +294,7 @@
     <t>Macabeo / Parellada / Xarello</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Freixenet%20Cordon%20Negro%20Brut.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Freixenet_Cordon_Negro_Brut-removebg-preview.avif</t>
   </si>
   <si>
     <t>Glenfiddich 15 anos Single Malt</t>
@@ -318,7 +318,7 @@
     <t>Single Malt</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Glenfiddich%2015%20anos%20Single%20Malt.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Glenfiddich_15_anos_Single_Malt-removebg-preview.avif</t>
   </si>
   <si>
     <t>Hendricks Gin</t>
@@ -339,7 +339,7 @@
     <t>Blend de botanicos</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Hendricks%20Gin.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Hendricks_Gin-removebg-preview.avif</t>
   </si>
   <si>
     <t>Hugel Riesling Classic</t>
@@ -357,7 +357,7 @@
     <t>Riesling</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Hugel%20Riesling%20Classic.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Hugel_Riesling_Classic-removebg-preview.avif</t>
   </si>
   <si>
     <t>Jack Daniels Old No. 7 Tennessee Whiskey</t>
@@ -378,7 +378,7 @@
     <t>Blend</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Jack%20Daniels%20Old%20No.%207%20Tennessee%20Whiskey.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Jack_Daniels_Old_No._7_Tennessee_Whiskey-removebg-preview.avif</t>
   </si>
   <si>
     <t>Johnnie Walker Black Label 12 anos</t>
@@ -393,7 +393,7 @@
     <t>Highlands / Speyside</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Johnnie%20Walker%20Black%20Label%2012%20anos.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Johnnie_Walker_Black_Label_12_anos-removebg-preview.avif</t>
   </si>
   <si>
     <t>Macallan 12 anos Sherry Oak</t>
@@ -405,7 +405,7 @@
     <t>Macallan</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Macallan%2012%20anos%20Sherry%20Oak.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Macallan_12_anos_Sherry_Oak-removebg-preview.avif</t>
   </si>
   <si>
     <t>Marques de Caceres Crianza Rioja</t>
@@ -423,7 +423,7 @@
     <t>Tempranillo</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Marques%20de%20Caceres%20Crianza%20Rioja.jpeg</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Marques_de_Caceres_Crianza_Rioja-removebg-preview.avif</t>
   </si>
   <si>
     <t>Moet and Chandon Brut Imperial</t>
@@ -441,7 +441,7 @@
     <t>Pinot Noir / Chardonnay / Meunier</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Moet%20and%20Chandon%20Brut%20Imperial.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Moet_and_Chandon_Brut_Imperial-removebg-preview.avif</t>
   </si>
   <si>
     <t>Montes Alpha Cabernet Sauvignon</t>
@@ -456,7 +456,7 @@
     <t>Valle de Colchagua</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Montes%20Alpha%20Cabernet%20Sauvignon.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Montes_Alpha_Cabernet_Sauvignon-removebg-preview.avif</t>
   </si>
   <si>
     <t>Patron Silver Tequila</t>
@@ -471,7 +471,7 @@
     <t>Jalisco / Highlands</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Patron%20Silver%20Tequila.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Patron_Silver_Tequila-removebg-preview.avif</t>
   </si>
   <si>
     <t>Penfolds Koonunga Hill Shiraz</t>
@@ -492,7 +492,7 @@
     <t>Shiraz</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Penfolds%20Koonunga%20Hill%20Shiraz.jpg</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Penfolds_Koonunga_Hill_Shiraz-removebg-preview.avif</t>
   </si>
   <si>
     <t>Santa Carolina Reserva Carmenere</t>
@@ -510,7 +510,7 @@
     <t>Carmenere</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Santa%20Carolina%20Reserva%20Carmenere.png</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Santa_Carolina_Reserva_Carmenere-removebg-preview.avif</t>
   </si>
   <si>
     <t>Santa Rita Reserva Sauvignon Blanc</t>
@@ -522,7 +522,7 @@
     <t>Santa Rita</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Santa%20Rita%20Reserva%20Sauvignon%20Blanc.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Santa_Rita_Reserva_Sauvignon_Blanc-removebg-preview.avif</t>
   </si>
   <si>
     <t>Torres Mas La Plana Cabernet Sauvignon</t>
@@ -537,7 +537,7 @@
     <t>Penedes</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Torres%20Mas%20La%20Plana%20Cabernet%20Sauvignon.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Torres_Mas_La_Plana_Cabernet_Sauvignon-removebg-preview.avif</t>
   </si>
   <si>
     <t>Torres Vina Esmeralda Moscatel</t>
@@ -549,7 +549,7 @@
     <t>Moscatel / Gewurztraminer</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Torres%20Vina%20Esmeralda%20Moscatel.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Torres_Vina_Esmeralda_Moscatel-removebg-preview.avif</t>
   </si>
   <si>
     <t>Trivento Golden Reserve Rose</t>
@@ -564,7 +564,7 @@
     <t>Trivento</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Trivento%20Golden%20Reserve%20Rose.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Trivento_Golden_Reserve_Rose-removebg-preview.avif</t>
   </si>
   <si>
     <t>Veuve Clicquot Yellow Label Brut</t>
@@ -579,7 +579,7 @@
     <t>Pinot Noir / Meunier / Chardonnay</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Veuve%20Clicquot%20Yellow%20Label%20Brut.jpeg</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Veuve_Clicquot_Yellow_Label_Brut-removebg-preview.avif</t>
   </si>
   <si>
     <t>Zacapa 23 Centenario</t>
@@ -597,7 +597,7 @@
     <t>Quetzaltenango</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Zacapa%2023%20Centenario.webp</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Zacapa_23_Centenario-removebg-preview.avif</t>
   </si>
   <si>
     <t>Zuccardi Valle de Uco Malbec</t>
@@ -606,7 +606,7 @@
     <t>Malbec de altura con notas de frutos negros y toques florales</t>
   </si>
   <si>
-    <t>https://storage.googleapis.com/tienda_vinos/Zuccardi%20Valle%20de%20Uco%20Malbec.jpeg</t>
+    <t>https://storage.googleapis.com/tienda_vinos/fotos_no_fondo/Zuccardi_Valle_de_Uco_Malbec-removebg-preview.avif</t>
   </si>
   <si>
     <t>ID,Nombre,Descripcion,Cantidad,Categoria,Subcategoria,Marca,Pais,Region,Cepa / Variedad,Anio Cosecha,Contenido (ml),Alcohol (%),Precio (USD),Descuento,Imagen,Estado</t>

</xml_diff>